<commit_message>
Add KWA board reporting and mixed-pressure runs
</commit_message>
<xml_diff>
--- a/data/knowledge_work/artifact_goldens/kwa_finance_three_statement_model__financial_model.xlsx
+++ b/data/knowledge_work/artifact_goldens/kwa_finance_three_statement_model__financial_model.xlsx
@@ -413,12 +413,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -444,6 +446,10 @@
           <t>Build a seeded three-statement-style operating view from filings and commentary.</t>
         </is>
       </c>
+      <c r="E2">
+        <f>BASE_REVENUE+DELTA</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -460,6 +466,10 @@
         <is>
           <t>Evidence</t>
         </is>
+      </c>
+      <c r="E3">
+        <f>BASE_EXPENSE+MARKETING_INCREASE</f>
+        <v/>
       </c>
     </row>
     <row r="4">

</xml_diff>